<commit_message>
The changes are commmited
</commit_message>
<xml_diff>
--- a/public/monthly_report.xlsx
+++ b/public/monthly_report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bharath/Documents/Innovative/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CB5E75E-A60D-0840-BFC6-ACA061144ECB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1D52C1E-668D-AB43-9283-81E4F1C4B13F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{10BE6AC1-B987-4FEE-A0F0-F452DA64378F}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="712" uniqueCount="294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="712" uniqueCount="295">
   <si>
     <t>Vinnovative Engineering Private Limited</t>
   </si>
@@ -919,6 +919,9 @@
   </si>
   <si>
     <t>142</t>
+  </si>
+  <si>
+    <t>Test</t>
   </si>
 </sst>
 </file>
@@ -1672,7 +1675,7 @@
         <v>53</v>
       </c>
       <c r="C9" s="35" t="s">
-        <v>56</v>
+        <v>294</v>
       </c>
       <c r="D9" s="36" t="s">
         <v>57</v>

</xml_diff>

<commit_message>
The excelsheet has updated
</commit_message>
<xml_diff>
--- a/public/monthly_report.xlsx
+++ b/public/monthly_report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bharath/Documents/Innovative/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1D52C1E-668D-AB43-9283-81E4F1C4B13F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42B374DF-AD86-A146-8F48-56416286F508}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{10BE6AC1-B987-4FEE-A0F0-F452DA64378F}"/>
   </bookViews>
@@ -921,7 +921,7 @@
     <t>142</t>
   </si>
   <si>
-    <t>Test</t>
+    <t>Update latest code</t>
   </si>
 </sst>
 </file>

</xml_diff>